<commit_message>
Int: Implemented metric / imperial prefs
</commit_message>
<xml_diff>
--- a/_devHelpers/DataClassHelper.xlsx
+++ b/_devHelpers/DataClassHelper.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter_old/HC/HarrierCentral/HarrierCentralMobile-Flutter/_devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F61D697-8BBC-FD4F-B266-2BF0F2C38931}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF3AC42-F93B-5A41-B35C-F4032561AE2B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-60160" yWindow="-17580" windowWidth="60160" windowHeight="33840" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
   <si>
     <t>wireName</t>
   </si>
@@ -76,13 +76,10 @@
     <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
   </si>
   <si>
-    <t>isKennelFollowing</t>
+    <t>distancePreference</t>
   </si>
   <si>
-    <t>mismanagementRoles</t>
-  </si>
-  <si>
-    <t>HasherKennelMapTableHelper</t>
+    <t>CountriesTableHelper</t>
   </si>
 </sst>
 </file>
@@ -496,7 +493,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>13</v>
@@ -511,115 +508,113 @@
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>isKennelFollowing</v>
+        <v>distancePreference</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.isKennelFollowing,</v>
+        <v>this.distancePreference,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final int isKennelFollowing;</v>
+        <v>final int distancePreference;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>isKennelFollowing: jsonItem['isKennelFollowing'],</v>
+        <v>distancePreference: jsonItem['distancePreference'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>IsKennelFollowing</v>
+        <v>DistancePreference</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colIsKennelFollowing</v>
+        <v>colDistancePreference</v>
       </c>
       <c r="I2" t="str">
         <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colIsKennelFollowing= 'isKennelFollowing';</v>
+        <v>static const String colDistancePreference= 'distancePreference';</v>
       </c>
       <c r="J2" t="str">
-        <f t="shared" ref="J2:J21" si="3">"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colIsKennelFollowing INT,</v>
+        <f>"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
+        <v>$colDistancePreference INT,</v>
       </c>
       <c r="K2" t="str">
-        <f t="shared" ref="K2:K21" si="4">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>HasherKennelMapTableHelper.colIsKennelFollowing: item.isKennelFollowing,</v>
+        <f t="shared" ref="K2:K21" si="3">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
+        <v>CountriesTableHelper.colDistancePreference: item.distancePreference,</v>
       </c>
       <c r="L2" t="str">
         <f>$K$1&amp;"."&amp;H2&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>HasherKennelMapTableHelper.colIsKennelFollowing: inputMap[HasherKennelMapTableHelper.colIsKennelFollowing],</v>
+        <v>CountriesTableHelper.colDistancePreference: inputMap[CountriesTableHelper.colDistancePreference],</v>
       </c>
       <c r="M2" t="str">
-        <f t="shared" ref="M2:M21" si="5">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>isKennelFollowing: map[HasherKennelMapTableHelper.colIsKennelFollowing],</v>
+        <f t="shared" ref="M2:M21" si="4">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
+        <v>distancePreference: map[CountriesTableHelper.colDistancePreference],</v>
       </c>
       <c r="N2" t="str">
         <f>"{ name: '"&amp;C2&amp;"', value: req.body."&amp;C2&amp;" },"</f>
-        <v>{ name: 'isKennelFollowing', value: req.body.isKennelFollowing },</v>
+        <v>{ name: 'distancePreference', value: req.body.distancePreference },</v>
       </c>
       <c r="O2" t="str">
         <f>"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H2&amp;"} "&amp;B2&amp;";"</f>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.colIsKennelFollowing} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.colDistancePreference} INT;</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C22" si="6">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
-        <v>mismanagementRoles</v>
+        <f t="shared" ref="C3:C22" si="5">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <f t="shared" ref="D3:D22" si="7">"this."&amp;C3 &amp; ","</f>
-        <v>this.mismanagementRoles,</v>
+        <f t="shared" ref="D3:D22" si="6">"this."&amp;C3 &amp; ","</f>
+        <v>this.,</v>
       </c>
       <c r="E3" t="str">
         <f>"final " &amp; VLOOKUP(B3,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C3 &amp; ";"</f>
-        <v>final int mismanagementRoles;</v>
+        <v>final int ;</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
-        <v>mismanagementRoles: jsonItem['mismanagementRoles'],</v>
+        <v>: jsonItem[''],</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
-        <v>MismanagementRoles</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H21" si="8">"col"&amp;G3</f>
-        <v>colMismanagementRoles</v>
+        <f t="shared" ref="H3:H21" si="7">"col"&amp;G3</f>
+        <v>col</v>
       </c>
       <c r="I3" t="str">
         <f t="shared" si="2"/>
-        <v>static const String colMismanagementRoles= 'mismanagementRoles';</v>
+        <v>static const String col= '';</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" si="3"/>
-        <v>$colMismanagementRoles INT,</v>
+        <f t="shared" ref="J2:J21" si="8">"$"&amp;H3&amp;" "&amp;B3&amp;","</f>
+        <v>$col INT,</v>
       </c>
       <c r="K3" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.colMismanagementRoles: item.mismanagementRoles,</v>
+        <f>$K$1&amp;"."&amp;H3&amp;": item."&amp;C3&amp;","</f>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" ref="L3:L21" si="9">$K$1&amp;"."&amp;H3&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H3&amp;"],"</f>
-        <v>HasherKennelMapTableHelper.colMismanagementRoles: inputMap[HasherKennelMapTableHelper.colMismanagementRoles],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M3" t="str">
-        <f t="shared" si="5"/>
-        <v>mismanagementRoles: map[HasherKennelMapTableHelper.colMismanagementRoles],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N3" t="str">
         <f t="shared" ref="N3:N21" si="10">"{ name: '"&amp;C3&amp;"', value: req.body."&amp;C3&amp;" },"</f>
-        <v>{ name: 'mismanagementRoles', value: req.body.mismanagementRoles },</v>
+        <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O3" t="str">
         <f t="shared" ref="O3:O21" si="11">"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H3&amp;"} "&amp;B3&amp;";"</f>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.colMismanagementRoles} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -628,11 +623,11 @@
         <v>4</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E4" t="str">
@@ -648,7 +643,7 @@
         <v/>
       </c>
       <c r="H4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I4" t="str">
@@ -656,20 +651,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K4" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M4" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N4" t="str">
         <f t="shared" si="10"/>
@@ -677,7 +672,7 @@
       </c>
       <c r="O4" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -686,11 +681,11 @@
         <v>5</v>
       </c>
       <c r="C5" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D5" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E5" t="str">
@@ -706,7 +701,7 @@
         <v/>
       </c>
       <c r="H5" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I5" t="str">
@@ -714,20 +709,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J5" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M5" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N5" t="str">
         <f t="shared" si="10"/>
@@ -735,7 +730,7 @@
       </c>
       <c r="O5" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -744,11 +739,11 @@
         <v>3</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E6" t="str">
@@ -764,7 +759,7 @@
         <v/>
       </c>
       <c r="H6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I6" t="str">
@@ -772,20 +767,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M6" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N6" t="str">
         <f t="shared" si="10"/>
@@ -793,7 +788,7 @@
       </c>
       <c r="O6" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -802,11 +797,11 @@
         <v>4</v>
       </c>
       <c r="C7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D7" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E7" t="str">
@@ -822,7 +817,7 @@
         <v/>
       </c>
       <c r="H7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I7" t="str">
@@ -830,20 +825,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M7" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N7" t="str">
         <f t="shared" si="10"/>
@@ -851,7 +846,7 @@
       </c>
       <c r="O7" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -860,11 +855,11 @@
         <v>4</v>
       </c>
       <c r="C8" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E8" t="str">
@@ -880,7 +875,7 @@
         <v/>
       </c>
       <c r="H8" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I8" t="str">
@@ -888,20 +883,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J8" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M8" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" si="10"/>
@@ -909,7 +904,7 @@
       </c>
       <c r="O8" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -918,11 +913,11 @@
         <v>4</v>
       </c>
       <c r="C9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E9" t="str">
@@ -938,7 +933,7 @@
         <v/>
       </c>
       <c r="H9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I9" t="str">
@@ -946,20 +941,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J9" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M9" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" si="10"/>
@@ -967,7 +962,7 @@
       </c>
       <c r="O9" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -976,11 +971,11 @@
         <v>5</v>
       </c>
       <c r="C10" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E10" t="str">
@@ -996,7 +991,7 @@
         <v/>
       </c>
       <c r="H10" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I10" t="str">
@@ -1004,20 +999,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J10" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M10" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" si="10"/>
@@ -1025,7 +1020,7 @@
       </c>
       <c r="O10" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -1034,11 +1029,11 @@
         <v>5</v>
       </c>
       <c r="C11" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E11" t="str">
@@ -1054,7 +1049,7 @@
         <v/>
       </c>
       <c r="H11" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I11" t="str">
@@ -1062,20 +1057,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M11" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" si="10"/>
@@ -1083,7 +1078,7 @@
       </c>
       <c r="O11" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1092,11 +1087,11 @@
         <v>4</v>
       </c>
       <c r="C12" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D12" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E12" t="str">
@@ -1112,7 +1107,7 @@
         <v/>
       </c>
       <c r="H12" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I12" t="str">
@@ -1120,20 +1115,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M12" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" si="10"/>
@@ -1141,7 +1136,7 @@
       </c>
       <c r="O12" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -1150,11 +1145,11 @@
         <v>3</v>
       </c>
       <c r="C13" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D13" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="E13" t="str">
@@ -1170,7 +1165,7 @@
         <v/>
       </c>
       <c r="H13" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I13" t="str">
@@ -1178,20 +1173,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M13" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" si="10"/>
@@ -1199,7 +1194,7 @@
       </c>
       <c r="O13" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -1207,11 +1202,11 @@
         <v>4</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F14" t="str">
@@ -1223,7 +1218,7 @@
         <v/>
       </c>
       <c r="H14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I14" t="str">
@@ -1231,20 +1226,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M14" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" si="10"/>
@@ -1252,7 +1247,7 @@
       </c>
       <c r="O14" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -1260,11 +1255,11 @@
         <v>5</v>
       </c>
       <c r="C15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F15" t="str">
@@ -1276,7 +1271,7 @@
         <v/>
       </c>
       <c r="H15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I15" t="str">
@@ -1284,20 +1279,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M15" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" si="10"/>
@@ -1305,7 +1300,7 @@
       </c>
       <c r="O15" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -1313,11 +1308,11 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D16" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F16" t="str">
@@ -1329,7 +1324,7 @@
         <v/>
       </c>
       <c r="H16" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I16" t="str">
@@ -1337,20 +1332,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M16" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" si="10"/>
@@ -1358,7 +1353,7 @@
       </c>
       <c r="O16" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.2">
@@ -1366,11 +1361,11 @@
         <v>5</v>
       </c>
       <c r="C17" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D17" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F17" t="str">
@@ -1382,7 +1377,7 @@
         <v/>
       </c>
       <c r="H17" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I17" t="str">
@@ -1390,20 +1385,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M17" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" si="10"/>
@@ -1411,7 +1406,7 @@
       </c>
       <c r="O17" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.2">
@@ -1419,11 +1414,11 @@
         <v>5</v>
       </c>
       <c r="C18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F18" t="str">
@@ -1435,7 +1430,7 @@
         <v/>
       </c>
       <c r="H18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I18" t="str">
@@ -1443,20 +1438,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col NUM,</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M18" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" si="10"/>
@@ -1464,7 +1459,7 @@
       </c>
       <c r="O18" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
@@ -1472,11 +1467,11 @@
         <v>3</v>
       </c>
       <c r="C19" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D19" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F19" t="str">
@@ -1488,7 +1483,7 @@
         <v/>
       </c>
       <c r="H19" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I19" t="str">
@@ -1496,20 +1491,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J19" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M19" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N19" t="str">
         <f t="shared" si="10"/>
@@ -1517,7 +1512,7 @@
       </c>
       <c r="O19" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.2">
@@ -1525,11 +1520,11 @@
         <v>3</v>
       </c>
       <c r="C20" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D20" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F20" t="str">
@@ -1541,7 +1536,7 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I20" t="str">
@@ -1549,20 +1544,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J20" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M20" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N20" t="str">
         <f t="shared" si="10"/>
@@ -1570,7 +1565,7 @@
       </c>
       <c r="O20" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
@@ -1578,11 +1573,11 @@
         <v>4</v>
       </c>
       <c r="C21" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D21" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
       <c r="F21" t="str">
@@ -1594,7 +1589,7 @@
         <v/>
       </c>
       <c r="H21" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>col</v>
       </c>
       <c r="I21" t="str">
@@ -1602,20 +1597,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J21" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>$col INT,</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="4"/>
-        <v>HasherKennelMapTableHelper.col: item.,</v>
+        <f t="shared" si="3"/>
+        <v>CountriesTableHelper.col: item.,</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="9"/>
-        <v>HasherKennelMapTableHelper.col: inputMap[HasherKennelMapTableHelper.col],</v>
+        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
       </c>
       <c r="M21" t="str">
-        <f t="shared" si="5"/>
-        <v>: map[HasherKennelMapTableHelper.col],</v>
+        <f t="shared" si="4"/>
+        <v>: map[CountriesTableHelper.col],</v>
       </c>
       <c r="N21" t="str">
         <f t="shared" si="10"/>
@@ -1623,16 +1618,16 @@
       </c>
       <c r="O21" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HasherKennelMapTableHelper.tableName} ADD COLUMN ${HasherKennelMapTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.2">
       <c r="C22" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="D22" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>this.,</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Int: Finished miles / km prefs
</commit_message>
<xml_diff>
--- a/_devHelpers/DataClassHelper.xlsx
+++ b/_devHelpers/DataClassHelper.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter_old/HC/HarrierCentral/HarrierCentralMobile-Flutter/_devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF3AC42-F93B-5A41-B35C-F4032561AE2B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6D9B2C-B5DD-6F42-BE34-3276EB774ABE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60160" yWindow="-17580" windowWidth="60160" windowHeight="33840" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -76,17 +76,17 @@
     <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
   </si>
   <si>
-    <t>distancePreference</t>
+    <t>preferences</t>
   </si>
   <si>
-    <t>CountriesTableHelper</t>
+    <t>HashersTableHelper</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -114,6 +114,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF4EC9B0"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -135,13 +141,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,6 +478,7 @@
     <col min="12" max="12" width="75.5" customWidth="1"/>
     <col min="13" max="13" width="61" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="74.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="90.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -492,7 +500,7 @@
       <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>15</v>
       </c>
       <c r="N1" s="2" t="s">
@@ -508,55 +516,55 @@
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>distancePreference</v>
+        <v>preferences</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.distancePreference,</v>
+        <v>this.preferences,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final int distancePreference;</v>
+        <v>final int preferences;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>distancePreference: jsonItem['distancePreference'],</v>
+        <v>preferences: jsonItem['preferences'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>DistancePreference</v>
+        <v>Preferences</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colDistancePreference</v>
+        <v>colPreferences</v>
       </c>
       <c r="I2" t="str">
         <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colDistancePreference= 'distancePreference';</v>
+        <v>static const String colPreferences= 'preferences';</v>
       </c>
       <c r="J2" t="str">
         <f>"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colDistancePreference INT,</v>
+        <v>$colPreferences INT,</v>
       </c>
       <c r="K2" t="str">
         <f t="shared" ref="K2:K21" si="3">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>CountriesTableHelper.colDistancePreference: item.distancePreference,</v>
+        <v>HashersTableHelper.colPreferences: item.preferences,</v>
       </c>
       <c r="L2" t="str">
         <f>$K$1&amp;"."&amp;H2&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>CountriesTableHelper.colDistancePreference: inputMap[CountriesTableHelper.colDistancePreference],</v>
+        <v>HashersTableHelper.colPreferences: inputMap[HashersTableHelper.colPreferences],</v>
       </c>
       <c r="M2" t="str">
         <f t="shared" ref="M2:M21" si="4">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>distancePreference: map[CountriesTableHelper.colDistancePreference],</v>
+        <v>preferences: map[HashersTableHelper.colPreferences],</v>
       </c>
       <c r="N2" t="str">
         <f>"{ name: '"&amp;C2&amp;"', value: req.body."&amp;C2&amp;" },"</f>
-        <v>{ name: 'distancePreference', value: req.body.distancePreference },</v>
+        <v>{ name: 'preferences', value: req.body.preferences },</v>
       </c>
       <c r="O2" t="str">
         <f>"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H2&amp;"} "&amp;B2&amp;";"</f>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.colDistancePreference} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.colPreferences} INT;</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -593,20 +601,20 @@
         <v>static const String col= '';</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J2:J21" si="8">"$"&amp;H3&amp;" "&amp;B3&amp;","</f>
+        <f t="shared" ref="J3:J21" si="8">"$"&amp;H3&amp;" "&amp;B3&amp;","</f>
         <v>$col INT,</v>
       </c>
       <c r="K3" t="str">
         <f>$K$1&amp;"."&amp;H3&amp;": item."&amp;C3&amp;","</f>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" ref="L3:L21" si="9">$K$1&amp;"."&amp;H3&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H3&amp;"],"</f>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M3" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N3" t="str">
         <f t="shared" ref="N3:N21" si="10">"{ name: '"&amp;C3&amp;"', value: req.body."&amp;C3&amp;" },"</f>
@@ -614,7 +622,7 @@
       </c>
       <c r="O3" t="str">
         <f t="shared" ref="O3:O21" si="11">"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H3&amp;"} "&amp;B3&amp;";"</f>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -656,15 +664,15 @@
       </c>
       <c r="K4" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M4" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N4" t="str">
         <f t="shared" si="10"/>
@@ -672,7 +680,7 @@
       </c>
       <c r="O4" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -714,15 +722,15 @@
       </c>
       <c r="K5" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M5" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N5" t="str">
         <f t="shared" si="10"/>
@@ -730,7 +738,7 @@
       </c>
       <c r="O5" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -772,15 +780,15 @@
       </c>
       <c r="K6" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M6" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N6" t="str">
         <f t="shared" si="10"/>
@@ -788,7 +796,7 @@
       </c>
       <c r="O6" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -830,15 +838,15 @@
       </c>
       <c r="K7" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M7" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N7" t="str">
         <f t="shared" si="10"/>
@@ -846,7 +854,7 @@
       </c>
       <c r="O7" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -888,15 +896,15 @@
       </c>
       <c r="K8" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M8" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" si="10"/>
@@ -904,7 +912,7 @@
       </c>
       <c r="O8" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -946,15 +954,15 @@
       </c>
       <c r="K9" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M9" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" si="10"/>
@@ -962,7 +970,7 @@
       </c>
       <c r="O9" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -1004,15 +1012,15 @@
       </c>
       <c r="K10" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M10" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" si="10"/>
@@ -1020,7 +1028,7 @@
       </c>
       <c r="O10" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -1062,15 +1070,15 @@
       </c>
       <c r="K11" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M11" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" si="10"/>
@@ -1078,7 +1086,7 @@
       </c>
       <c r="O11" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1120,15 +1128,15 @@
       </c>
       <c r="K12" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M12" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" si="10"/>
@@ -1136,7 +1144,7 @@
       </c>
       <c r="O12" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -1178,15 +1186,15 @@
       </c>
       <c r="K13" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M13" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" si="10"/>
@@ -1194,7 +1202,7 @@
       </c>
       <c r="O13" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -1231,15 +1239,15 @@
       </c>
       <c r="K14" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L14" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M14" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" si="10"/>
@@ -1247,7 +1255,7 @@
       </c>
       <c r="O14" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -1284,15 +1292,15 @@
       </c>
       <c r="K15" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M15" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" si="10"/>
@@ -1300,7 +1308,7 @@
       </c>
       <c r="O15" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -1337,15 +1345,15 @@
       </c>
       <c r="K16" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M16" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" si="10"/>
@@ -1353,7 +1361,7 @@
       </c>
       <c r="O16" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.2">
@@ -1390,15 +1398,15 @@
       </c>
       <c r="K17" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M17" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" si="10"/>
@@ -1406,7 +1414,7 @@
       </c>
       <c r="O17" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.2">
@@ -1443,15 +1451,15 @@
       </c>
       <c r="K18" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M18" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" si="10"/>
@@ -1459,7 +1467,7 @@
       </c>
       <c r="O18" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} NUM;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
@@ -1496,15 +1504,15 @@
       </c>
       <c r="K19" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M19" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N19" t="str">
         <f t="shared" si="10"/>
@@ -1512,7 +1520,7 @@
       </c>
       <c r="O19" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.2">
@@ -1549,15 +1557,15 @@
       </c>
       <c r="K20" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L20" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M20" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N20" t="str">
         <f t="shared" si="10"/>
@@ -1565,7 +1573,7 @@
       </c>
       <c r="O20" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} TEXT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
@@ -1602,15 +1610,15 @@
       </c>
       <c r="K21" t="str">
         <f t="shared" si="3"/>
-        <v>CountriesTableHelper.col: item.,</v>
+        <v>HashersTableHelper.col: item.,</v>
       </c>
       <c r="L21" t="str">
         <f t="shared" si="9"/>
-        <v>CountriesTableHelper.col: inputMap[CountriesTableHelper.col],</v>
+        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
       </c>
       <c r="M21" t="str">
         <f t="shared" si="4"/>
-        <v>: map[CountriesTableHelper.col],</v>
+        <v>: map[HashersTableHelper.col],</v>
       </c>
       <c r="N21" t="str">
         <f t="shared" si="10"/>
@@ -1618,7 +1626,7 @@
       </c>
       <c r="O21" t="str">
         <f t="shared" si="11"/>
-        <v>ALTER TABLE ${CountriesTableHelper.tableName} ADD COLUMN ${CountriesTableHelper.col} INT;</v>
+        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Int: added region & subRegion to internal db
</commit_message>
<xml_diff>
--- a/_devHelpers/DataClassHelper.xlsx
+++ b/_devHelpers/DataClassHelper.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameswhite/Projects/flutter_old/HC/HarrierCentral/HarrierCentralMobile-Flutter/_devHelpers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6D9B2C-B5DD-6F42-BE34-3276EB774ABE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F307A42F-6EC4-C54E-84E5-55CFFFA855DF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="20540" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
+    <workbookView xWindow="-27320" yWindow="-11000" windowWidth="27320" windowHeight="20480" xr2:uid="{50A37692-8663-7F4C-91F6-2AE3BA380A00}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="17">
   <si>
     <t>wireName</t>
   </si>
@@ -76,10 +78,13 @@
     <t>{ name: 'receiptAmount', value: req.body.receiptAmount },</t>
   </si>
   <si>
-    <t>preferences</t>
+    <t>locationRegion</t>
   </si>
   <si>
-    <t>HashersTableHelper</t>
+    <t>locationSubRegion</t>
+  </si>
+  <si>
+    <t>eventsTableHelper</t>
   </si>
 </sst>
 </file>
@@ -500,11 +505,11 @@
       <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
-        <v>15</v>
-      </c>
       <c r="N1" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -512,117 +517,119 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="str">
         <f>SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A2," ",REPT(" ",100)),100)),",","")</f>
-        <v>preferences</v>
+        <v>locationRegion</v>
       </c>
       <c r="D2" t="str">
         <f>"this."&amp;C2 &amp; ","</f>
-        <v>this.preferences,</v>
+        <v>this.locationRegion,</v>
       </c>
       <c r="E2" t="str">
         <f>"final " &amp; VLOOKUP(B2,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C2 &amp; ";"</f>
-        <v>final int preferences;</v>
+        <v>final String locationRegion;</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F21" si="0">C2&amp;": jsonItem['"&amp;C2&amp;"'],"</f>
-        <v>preferences: jsonItem['preferences'],</v>
+        <v>locationRegion: jsonItem['locationRegion'],</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G21" si="1">UPPER(MID(C2,1,1)) &amp; MID(C2,2,9999)</f>
-        <v>Preferences</v>
+        <v>LocationRegion</v>
       </c>
       <c r="H2" t="str">
         <f>"col"&amp;G2</f>
-        <v>colPreferences</v>
+        <v>colLocationRegion</v>
       </c>
       <c r="I2" t="str">
-        <f t="shared" ref="I2:I21" si="2">"static const String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
-        <v>static const String colPreferences= 'preferences';</v>
+        <f>"final String "&amp;H2&amp;"= '"&amp;C2&amp;"';"</f>
+        <v>final String colLocationRegion= 'locationRegion';</v>
       </c>
       <c r="J2" t="str">
         <f>"$"&amp;H2&amp;" "&amp;B2&amp;","</f>
-        <v>$colPreferences INT,</v>
+        <v>$colLocationRegion TEXT,</v>
       </c>
       <c r="K2" t="str">
-        <f t="shared" ref="K2:K21" si="3">$K$1&amp;"."&amp;H2&amp;": item."&amp;C2&amp;","</f>
-        <v>HashersTableHelper.colPreferences: item.preferences,</v>
+        <f>H2&amp;": item."&amp;C2&amp;","</f>
+        <v>colLocationRegion: item.locationRegion,</v>
       </c>
       <c r="L2" t="str">
-        <f>$K$1&amp;"."&amp;H2&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>HashersTableHelper.colPreferences: inputMap[HashersTableHelper.colPreferences],</v>
+        <f>H2&amp;": "&amp;"inputMap["&amp;H2&amp;"],"</f>
+        <v>colLocationRegion: inputMap[colLocationRegion],</v>
       </c>
       <c r="M2" t="str">
-        <f t="shared" ref="M2:M21" si="4">C2&amp;": map["&amp;$K$1&amp;"."&amp;H2&amp;"],"</f>
-        <v>preferences: map[HashersTableHelper.colPreferences],</v>
+        <f>C2&amp;": map["&amp;H2&amp;"],"</f>
+        <v>locationRegion: map[colLocationRegion],</v>
       </c>
       <c r="N2" t="str">
         <f>"{ name: '"&amp;C2&amp;"', value: req.body."&amp;C2&amp;" },"</f>
-        <v>{ name: 'preferences', value: req.body.preferences },</v>
+        <v>{ name: 'locationRegion', value: req.body.locationRegion },</v>
       </c>
       <c r="O2" t="str">
-        <f>"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H2&amp;"} "&amp;B2&amp;";"</f>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.colPreferences} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H2&amp;"} "&amp;B2&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.colLocationRegion} TEXT;</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C22" si="5">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
-        <v/>
+        <f t="shared" ref="C3:C22" si="2">SUBSTITUTE(TRIM(RIGHT(SUBSTITUTE(A3," ",REPT(" ",100)),100)),",","")</f>
+        <v>locationSubRegion</v>
       </c>
       <c r="D3" t="str">
-        <f t="shared" ref="D3:D22" si="6">"this."&amp;C3 &amp; ","</f>
-        <v>this.,</v>
+        <f t="shared" ref="D3:D22" si="3">"this."&amp;C3 &amp; ","</f>
+        <v>this.locationSubRegion,</v>
       </c>
       <c r="E3" t="str">
         <f>"final " &amp; VLOOKUP(B3,Sheet2!$A$1:$B$4,2,FALSE) &amp; " " &amp; C3 &amp; ";"</f>
-        <v>final int ;</v>
+        <v>final String locationSubRegion;</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
-        <v>: jsonItem[''],</v>
+        <v>locationSubRegion: jsonItem['locationSubRegion'],</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>LocationSubRegion</v>
       </c>
       <c r="H3" t="str">
-        <f t="shared" ref="H3:H21" si="7">"col"&amp;G3</f>
-        <v>col</v>
+        <f t="shared" ref="H3:H21" si="4">"col"&amp;G3</f>
+        <v>colLocationSubRegion</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" ref="I3:I21" si="5">"final String "&amp;H3&amp;"= '"&amp;C3&amp;"';"</f>
+        <v>final String colLocationSubRegion= 'locationSubRegion';</v>
       </c>
       <c r="J3" t="str">
-        <f t="shared" ref="J3:J21" si="8">"$"&amp;H3&amp;" "&amp;B3&amp;","</f>
-        <v>$col INT,</v>
+        <f t="shared" ref="J3:J21" si="6">"$"&amp;H3&amp;" "&amp;B3&amp;","</f>
+        <v>$colLocationSubRegion TEXT,</v>
       </c>
       <c r="K3" t="str">
-        <f>$K$1&amp;"."&amp;H3&amp;": item."&amp;C3&amp;","</f>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" ref="K3:K21" si="7">H3&amp;": item."&amp;C3&amp;","</f>
+        <v>colLocationSubRegion: item.locationSubRegion,</v>
       </c>
       <c r="L3" t="str">
-        <f t="shared" ref="L3:L21" si="9">$K$1&amp;"."&amp;H3&amp;": "&amp;"inputMap["&amp;$K$1&amp;"."&amp;H3&amp;"],"</f>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" ref="L3:L21" si="8">H3&amp;": "&amp;"inputMap["&amp;H3&amp;"],"</f>
+        <v>colLocationSubRegion: inputMap[colLocationSubRegion],</v>
       </c>
       <c r="M3" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" ref="M3:M21" si="9">C3&amp;": map["&amp;H3&amp;"],"</f>
+        <v>locationSubRegion: map[colLocationSubRegion],</v>
       </c>
       <c r="N3" t="str">
         <f t="shared" ref="N3:N21" si="10">"{ name: '"&amp;C3&amp;"', value: req.body."&amp;C3&amp;" },"</f>
-        <v>{ name: '', value: req.body. },</v>
+        <v>{ name: 'locationSubRegion', value: req.body.locationSubRegion },</v>
       </c>
       <c r="O3" t="str">
-        <f t="shared" ref="O3:O21" si="11">"ALTER TABLE ${"&amp;$K$1&amp;".tableName} ADD COLUMN ${"&amp;$K$1&amp;"."&amp;H3&amp;"} "&amp;B3&amp;";"</f>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H3&amp;"} "&amp;B3&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.colLocationSubRegion} TEXT;</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -631,11 +638,11 @@
         <v>4</v>
       </c>
       <c r="C4" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D4" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E4" t="str">
@@ -651,36 +658,36 @@
         <v/>
       </c>
       <c r="H4" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I4" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J4" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K4" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L4" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M4" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N4" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O4" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H4&amp;"} "&amp;B4&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -689,11 +696,11 @@
         <v>5</v>
       </c>
       <c r="C5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D5" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E5" t="str">
@@ -709,36 +716,36 @@
         <v/>
       </c>
       <c r="H5" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I5" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J5" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L5" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M5" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N5" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O5" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H5&amp;"} "&amp;B5&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -747,11 +754,11 @@
         <v>3</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D6" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E6" t="str">
@@ -767,36 +774,36 @@
         <v/>
       </c>
       <c r="H6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I6" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J6" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L6" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M6" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N6" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O6" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H6&amp;"} "&amp;B6&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -805,11 +812,11 @@
         <v>4</v>
       </c>
       <c r="C7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E7" t="str">
@@ -825,36 +832,36 @@
         <v/>
       </c>
       <c r="H7" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I7" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J7" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L7" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M7" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N7" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O7" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H7&amp;"} "&amp;B7&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -863,11 +870,11 @@
         <v>4</v>
       </c>
       <c r="C8" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D8" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E8" t="str">
@@ -883,36 +890,36 @@
         <v/>
       </c>
       <c r="H8" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I8" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J8" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L8" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M8" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O8" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H8&amp;"} "&amp;B8&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -921,11 +928,11 @@
         <v>4</v>
       </c>
       <c r="C9" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E9" t="str">
@@ -941,36 +948,36 @@
         <v/>
       </c>
       <c r="H9" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I9" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L9" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M9" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O9" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H9&amp;"} "&amp;B9&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -979,11 +986,11 @@
         <v>5</v>
       </c>
       <c r="C10" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D10" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E10" t="str">
@@ -999,36 +1006,36 @@
         <v/>
       </c>
       <c r="H10" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I10" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J10" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L10" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M10" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O10" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H10&amp;"} "&amp;B10&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -1037,11 +1044,11 @@
         <v>5</v>
       </c>
       <c r="C11" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D11" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E11" t="str">
@@ -1057,36 +1064,36 @@
         <v/>
       </c>
       <c r="H11" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I11" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J11" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L11" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M11" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O11" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H11&amp;"} "&amp;B11&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -1095,11 +1102,11 @@
         <v>4</v>
       </c>
       <c r="C12" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D12" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E12" t="str">
@@ -1115,36 +1122,36 @@
         <v/>
       </c>
       <c r="H12" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I12" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J12" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L12" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M12" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O12" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H12&amp;"} "&amp;B12&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -1153,11 +1160,11 @@
         <v>3</v>
       </c>
       <c r="C13" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D13" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="E13" t="str">
@@ -1173,36 +1180,36 @@
         <v/>
       </c>
       <c r="H13" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I13" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J13" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L13" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M13" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O13" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H13&amp;"} "&amp;B13&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -1210,11 +1217,11 @@
         <v>4</v>
       </c>
       <c r="C14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F14" t="str">
@@ -1226,36 +1233,36 @@
         <v/>
       </c>
       <c r="H14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I14" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J14" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L14" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M14" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N14" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O14" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H14&amp;"} "&amp;B14&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -1263,11 +1270,11 @@
         <v>5</v>
       </c>
       <c r="C15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F15" t="str">
@@ -1279,36 +1286,36 @@
         <v/>
       </c>
       <c r="H15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I15" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J15" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L15" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M15" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O15" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H15&amp;"} "&amp;B15&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -1316,11 +1323,11 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D16" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F16" t="str">
@@ -1332,36 +1339,36 @@
         <v/>
       </c>
       <c r="H16" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I16" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J16" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L16" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M16" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O16" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H16&amp;"} "&amp;B16&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.2">
@@ -1369,11 +1376,11 @@
         <v>5</v>
       </c>
       <c r="C17" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D17" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F17" t="str">
@@ -1385,36 +1392,36 @@
         <v/>
       </c>
       <c r="H17" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I17" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J17" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L17" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M17" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O17" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H17&amp;"} "&amp;B17&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.2">
@@ -1422,11 +1429,11 @@
         <v>5</v>
       </c>
       <c r="C18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F18" t="str">
@@ -1438,36 +1445,36 @@
         <v/>
       </c>
       <c r="H18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I18" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col NUM,</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L18" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M18" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O18" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} NUM;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H18&amp;"} "&amp;B18&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} NUM;</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
@@ -1475,11 +1482,11 @@
         <v>3</v>
       </c>
       <c r="C19" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D19" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F19" t="str">
@@ -1491,36 +1498,36 @@
         <v/>
       </c>
       <c r="H19" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I19" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J19" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L19" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M19" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N19" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O19" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H19&amp;"} "&amp;B19&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.2">
@@ -1528,11 +1535,11 @@
         <v>3</v>
       </c>
       <c r="C20" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D20" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F20" t="str">
@@ -1544,36 +1551,36 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I20" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J20" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col TEXT,</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L20" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M20" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N20" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O20" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} TEXT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H20&amp;"} "&amp;B20&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} TEXT;</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
@@ -1581,11 +1588,11 @@
         <v>4</v>
       </c>
       <c r="C21" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D21" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
       <c r="F21" t="str">
@@ -1597,50 +1604,51 @@
         <v/>
       </c>
       <c r="H21" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="4"/>
         <v>col</v>
       </c>
       <c r="I21" t="str">
-        <f t="shared" si="2"/>
-        <v>static const String col= '';</v>
+        <f t="shared" si="5"/>
+        <v>final String col= '';</v>
       </c>
       <c r="J21" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>$col INT,</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="3"/>
-        <v>HashersTableHelper.col: item.,</v>
+        <f t="shared" si="7"/>
+        <v>col: item.,</v>
       </c>
       <c r="L21" t="str">
-        <f t="shared" si="9"/>
-        <v>HashersTableHelper.col: inputMap[HashersTableHelper.col],</v>
+        <f t="shared" si="8"/>
+        <v>col: inputMap[col],</v>
       </c>
       <c r="M21" t="str">
-        <f t="shared" si="4"/>
-        <v>: map[HashersTableHelper.col],</v>
+        <f t="shared" si="9"/>
+        <v>: map[col],</v>
       </c>
       <c r="N21" t="str">
         <f t="shared" si="10"/>
         <v>{ name: '', value: req.body. },</v>
       </c>
       <c r="O21" t="str">
-        <f t="shared" si="11"/>
-        <v>ALTER TABLE ${HashersTableHelper.tableName} ADD COLUMN ${HashersTableHelper.col} INT;</v>
+        <f>"ALTER TABLE ${"&amp;$O$1&amp;".tableName} ADD COLUMN ${"&amp;$O$1&amp;"."&amp;H21&amp;"} "&amp;B21&amp;";"</f>
+        <v>ALTER TABLE ${eventsTableHelper.tableName} ADD COLUMN ${eventsTableHelper.col} INT;</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.2">
       <c r="C22" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="D22" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>this.,</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>